<commit_message>
ingesta: snapshot 2026-08-07 19:02 UTC
</commit_message>
<xml_diff>
--- a/data_lake/acumulado_tempmax_mes/dt=2026-08-07/Temp-max-agosto-26.xlsx
+++ b/data_lake/acumulado_tempmax_mes/dt=2026-08-07/Temp-max-agosto-26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.187.8\Oficina\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6506C524-C038-491F-BD36-3DE1DDAD82EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDC53C8-ACA5-4A0A-812A-9544224E245E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TMAX_PRINCIPALES_CIUDADES" sheetId="1" r:id="rId1"/>
@@ -9428,7 +9428,9 @@
       <c r="I5" s="63">
         <v>31.4</v>
       </c>
-      <c r="J5" s="63"/>
+      <c r="J5" s="63">
+        <v>31.6</v>
+      </c>
       <c r="K5" s="63"/>
       <c r="L5" s="63"/>
       <c r="M5" s="63"/>
@@ -9456,7 +9458,7 @@
       <c r="AI5" s="63"/>
       <c r="AJ5" s="36">
         <f>+IF(SUM($E5:$AI5)&gt;0,LOOKUP(1000,$E5:$AI5),NA())</f>
-        <v>31.4</v>
+        <v>31.6</v>
       </c>
       <c r="AK5" s="21">
         <f>+MAX($E5:$AI5)</f>
@@ -9509,7 +9511,9 @@
       <c r="I6" s="63">
         <v>31.2</v>
       </c>
-      <c r="J6" s="63"/>
+      <c r="J6" s="63">
+        <v>31.2</v>
+      </c>
       <c r="K6" s="63"/>
       <c r="L6" s="63"/>
       <c r="M6" s="63"/>
@@ -9590,7 +9594,9 @@
       <c r="I7" s="63">
         <v>34.200000000000003</v>
       </c>
-      <c r="J7" s="63"/>
+      <c r="J7" s="63">
+        <v>33.799999999999997</v>
+      </c>
       <c r="K7" s="63"/>
       <c r="L7" s="63"/>
       <c r="M7" s="63"/>
@@ -9618,7 +9624,7 @@
       <c r="AI7" s="63"/>
       <c r="AJ7" s="36">
         <f t="shared" si="0"/>
-        <v>34.200000000000003</v>
+        <v>33.799999999999997</v>
       </c>
       <c r="AK7" s="21">
         <f t="shared" si="1"/>
@@ -9671,7 +9677,9 @@
       <c r="I8" s="63">
         <v>33.299999999999997</v>
       </c>
-      <c r="J8" s="63"/>
+      <c r="J8" s="63">
+        <v>32.5</v>
+      </c>
       <c r="K8" s="63"/>
       <c r="L8" s="63"/>
       <c r="M8" s="63"/>
@@ -9699,7 +9707,7 @@
       <c r="AI8" s="63"/>
       <c r="AJ8" s="36">
         <f t="shared" si="0"/>
-        <v>33.299999999999997</v>
+        <v>32.5</v>
       </c>
       <c r="AK8" s="21">
         <f t="shared" si="1"/>
@@ -9752,7 +9760,9 @@
       <c r="I9" s="63">
         <v>34.9</v>
       </c>
-      <c r="J9" s="63"/>
+      <c r="J9" s="63">
+        <v>33.6</v>
+      </c>
       <c r="K9" s="63"/>
       <c r="L9" s="63"/>
       <c r="M9" s="63"/>
@@ -9780,7 +9790,7 @@
       <c r="AI9" s="63"/>
       <c r="AJ9" s="36">
         <f t="shared" si="0"/>
-        <v>34.9</v>
+        <v>33.6</v>
       </c>
       <c r="AK9" s="21">
         <f t="shared" si="1"/>
@@ -9833,7 +9843,9 @@
       <c r="I10" s="63">
         <v>35.200000000000003</v>
       </c>
-      <c r="J10" s="63"/>
+      <c r="J10" s="63">
+        <v>35.700000000000003</v>
+      </c>
       <c r="K10" s="63"/>
       <c r="L10" s="63"/>
       <c r="M10" s="63"/>
@@ -9861,7 +9873,7 @@
       <c r="AI10" s="63"/>
       <c r="AJ10" s="36">
         <f t="shared" si="0"/>
-        <v>35.200000000000003</v>
+        <v>35.700000000000003</v>
       </c>
       <c r="AK10" s="21">
         <f t="shared" si="1"/>
@@ -9914,7 +9926,9 @@
       <c r="I11" s="63">
         <v>37.700000000000003</v>
       </c>
-      <c r="J11" s="63"/>
+      <c r="J11" s="63">
+        <v>36.299999999999997</v>
+      </c>
       <c r="K11" s="63"/>
       <c r="L11" s="63"/>
       <c r="M11" s="63"/>
@@ -9942,7 +9956,7 @@
       <c r="AI11" s="63"/>
       <c r="AJ11" s="36">
         <f t="shared" si="0"/>
-        <v>37.700000000000003</v>
+        <v>36.299999999999997</v>
       </c>
       <c r="AK11" s="21">
         <f t="shared" si="1"/>
@@ -9995,7 +10009,9 @@
       <c r="I12" s="63">
         <v>35</v>
       </c>
-      <c r="J12" s="63"/>
+      <c r="J12" s="63">
+        <v>27.8</v>
+      </c>
       <c r="K12" s="63"/>
       <c r="L12" s="63"/>
       <c r="M12" s="63"/>
@@ -10023,7 +10039,7 @@
       <c r="AI12" s="63"/>
       <c r="AJ12" s="36">
         <f t="shared" si="0"/>
-        <v>35</v>
+        <v>27.8</v>
       </c>
       <c r="AK12" s="21">
         <f t="shared" si="1"/>
@@ -10076,7 +10092,9 @@
       <c r="I13" s="63">
         <v>34.4</v>
       </c>
-      <c r="J13" s="63"/>
+      <c r="J13" s="63">
+        <v>28.4</v>
+      </c>
       <c r="K13" s="63"/>
       <c r="L13" s="63"/>
       <c r="M13" s="63"/>
@@ -10104,7 +10122,7 @@
       <c r="AI13" s="63"/>
       <c r="AJ13" s="36">
         <f t="shared" si="0"/>
-        <v>34.4</v>
+        <v>28.4</v>
       </c>
       <c r="AK13" s="21">
         <f t="shared" si="1"/>
@@ -10157,7 +10175,9 @@
       <c r="I14" s="63">
         <v>35.6</v>
       </c>
-      <c r="J14" s="63"/>
+      <c r="J14" s="63">
+        <v>27.8</v>
+      </c>
       <c r="K14" s="63"/>
       <c r="L14" s="63"/>
       <c r="M14" s="63"/>
@@ -10185,7 +10205,7 @@
       <c r="AI14" s="63"/>
       <c r="AJ14" s="36">
         <f t="shared" si="0"/>
-        <v>35.6</v>
+        <v>27.8</v>
       </c>
       <c r="AK14" s="21">
         <f t="shared" si="1"/>
@@ -10238,7 +10258,9 @@
       <c r="I15" s="63">
         <v>31.8</v>
       </c>
-      <c r="J15" s="63"/>
+      <c r="J15" s="63">
+        <v>26.8</v>
+      </c>
       <c r="K15" s="63"/>
       <c r="L15" s="63"/>
       <c r="M15" s="63"/>
@@ -10266,7 +10288,7 @@
       <c r="AI15" s="63"/>
       <c r="AJ15" s="36">
         <f t="shared" si="0"/>
-        <v>31.8</v>
+        <v>26.8</v>
       </c>
       <c r="AK15" s="21">
         <f t="shared" si="1"/>
@@ -10368,7 +10390,9 @@
       <c r="I17" s="63">
         <v>35</v>
       </c>
-      <c r="J17" s="63"/>
+      <c r="J17" s="63">
+        <v>33.299999999999997</v>
+      </c>
       <c r="K17" s="63"/>
       <c r="L17" s="63"/>
       <c r="M17" s="63"/>
@@ -10396,7 +10420,7 @@
       <c r="AI17" s="63"/>
       <c r="AJ17" s="36">
         <f t="shared" si="0"/>
-        <v>35</v>
+        <v>33.299999999999997</v>
       </c>
       <c r="AK17" s="21">
         <f t="shared" si="1"/>
@@ -10449,7 +10473,9 @@
       <c r="I18" s="63">
         <v>28.2</v>
       </c>
-      <c r="J18" s="63"/>
+      <c r="J18" s="63">
+        <v>26.8</v>
+      </c>
       <c r="K18" s="63"/>
       <c r="L18" s="63"/>
       <c r="M18" s="63"/>
@@ -10477,7 +10503,7 @@
       <c r="AI18" s="63"/>
       <c r="AJ18" s="36">
         <f t="shared" si="0"/>
-        <v>28.2</v>
+        <v>26.8</v>
       </c>
       <c r="AK18" s="21">
         <f t="shared" si="1"/>
@@ -10530,7 +10556,9 @@
       <c r="I19" s="63">
         <v>34.700000000000003</v>
       </c>
-      <c r="J19" s="63"/>
+      <c r="J19" s="63">
+        <v>33.299999999999997</v>
+      </c>
       <c r="K19" s="63"/>
       <c r="L19" s="63"/>
       <c r="M19" s="63"/>
@@ -10558,7 +10586,7 @@
       <c r="AI19" s="63"/>
       <c r="AJ19" s="36">
         <f t="shared" si="0"/>
-        <v>34.700000000000003</v>
+        <v>33.299999999999997</v>
       </c>
       <c r="AK19" s="21">
         <f t="shared" si="1"/>
@@ -10611,7 +10639,9 @@
       <c r="I20" s="63">
         <v>29.5</v>
       </c>
-      <c r="J20" s="63"/>
+      <c r="J20" s="63">
+        <v>29.1</v>
+      </c>
       <c r="K20" s="63"/>
       <c r="L20" s="63"/>
       <c r="M20" s="63"/>
@@ -10639,7 +10669,7 @@
       <c r="AI20" s="63"/>
       <c r="AJ20" s="36">
         <f t="shared" si="0"/>
-        <v>29.5</v>
+        <v>29.1</v>
       </c>
       <c r="AK20" s="21">
         <f t="shared" si="1"/>
@@ -10692,7 +10722,9 @@
       <c r="I21" s="63">
         <v>23.3</v>
       </c>
-      <c r="J21" s="63"/>
+      <c r="J21" s="63">
+        <v>23.4</v>
+      </c>
       <c r="K21" s="63"/>
       <c r="L21" s="63"/>
       <c r="M21" s="63"/>
@@ -10720,7 +10752,7 @@
       <c r="AI21" s="63"/>
       <c r="AJ21" s="36">
         <f t="shared" si="0"/>
-        <v>23.3</v>
+        <v>23.4</v>
       </c>
       <c r="AK21" s="21">
         <f t="shared" si="1"/>
@@ -10841,7 +10873,9 @@
       <c r="I23" s="63">
         <v>26</v>
       </c>
-      <c r="J23" s="63"/>
+      <c r="J23" s="63">
+        <v>27.5</v>
+      </c>
       <c r="K23" s="63"/>
       <c r="L23" s="63"/>
       <c r="M23" s="63"/>
@@ -10869,7 +10903,7 @@
       <c r="AI23" s="63"/>
       <c r="AJ23" s="36">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>27.5</v>
       </c>
       <c r="AK23" s="21">
         <f t="shared" si="1"/>
@@ -10922,7 +10956,9 @@
       <c r="I24" s="63">
         <v>27</v>
       </c>
-      <c r="J24" s="63"/>
+      <c r="J24" s="63">
+        <v>27.5</v>
+      </c>
       <c r="K24" s="63"/>
       <c r="L24" s="63"/>
       <c r="M24" s="63"/>
@@ -10950,7 +10986,7 @@
       <c r="AI24" s="63"/>
       <c r="AJ24" s="36">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>27.5</v>
       </c>
       <c r="AK24" s="21">
         <f t="shared" si="1"/>
@@ -11003,7 +11039,9 @@
       <c r="I25" s="63">
         <v>29.9</v>
       </c>
-      <c r="J25" s="63"/>
+      <c r="J25" s="63">
+        <v>35.799999999999997</v>
+      </c>
       <c r="K25" s="63"/>
       <c r="L25" s="63"/>
       <c r="M25" s="63"/>
@@ -11031,7 +11069,7 @@
       <c r="AI25" s="63"/>
       <c r="AJ25" s="36">
         <f t="shared" si="0"/>
-        <v>29.9</v>
+        <v>35.799999999999997</v>
       </c>
       <c r="AK25" s="21">
         <f t="shared" si="1"/>
@@ -11084,7 +11122,9 @@
       <c r="I26" s="63">
         <v>18.399999999999999</v>
       </c>
-      <c r="J26" s="63"/>
+      <c r="J26" s="63">
+        <v>18.3</v>
+      </c>
       <c r="K26" s="63"/>
       <c r="L26" s="63"/>
       <c r="M26" s="63"/>
@@ -11112,7 +11152,7 @@
       <c r="AI26" s="63"/>
       <c r="AJ26" s="36">
         <f t="shared" si="0"/>
-        <v>18.399999999999999</v>
+        <v>18.3</v>
       </c>
       <c r="AK26" s="21">
         <f t="shared" si="1"/>
@@ -11165,7 +11205,9 @@
       <c r="I27" s="63">
         <v>18.2</v>
       </c>
-      <c r="J27" s="63"/>
+      <c r="J27" s="63">
+        <v>19.600000000000001</v>
+      </c>
       <c r="K27" s="63"/>
       <c r="L27" s="63"/>
       <c r="M27" s="63"/>
@@ -11193,7 +11235,7 @@
       <c r="AI27" s="63"/>
       <c r="AJ27" s="36">
         <f t="shared" si="0"/>
-        <v>18.2</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="AK27" s="21">
         <f t="shared" si="1"/>
@@ -11246,7 +11288,9 @@
       <c r="I28" s="63">
         <v>29.2</v>
       </c>
-      <c r="J28" s="63"/>
+      <c r="J28" s="63">
+        <v>31.3</v>
+      </c>
       <c r="K28" s="63"/>
       <c r="L28" s="63"/>
       <c r="M28" s="63"/>
@@ -11274,7 +11318,7 @@
       <c r="AI28" s="63"/>
       <c r="AJ28" s="36">
         <f t="shared" si="0"/>
-        <v>29.2</v>
+        <v>31.3</v>
       </c>
       <c r="AK28" s="21">
         <f t="shared" si="1"/>
@@ -11393,7 +11437,9 @@
       <c r="I30" s="63">
         <v>33.5</v>
       </c>
-      <c r="J30" s="63"/>
+      <c r="J30" s="63">
+        <v>35.4</v>
+      </c>
       <c r="K30" s="63"/>
       <c r="L30" s="63"/>
       <c r="M30" s="63"/>
@@ -11421,7 +11467,7 @@
       <c r="AI30" s="63"/>
       <c r="AJ30" s="36">
         <f t="shared" si="0"/>
-        <v>33.5</v>
+        <v>35.4</v>
       </c>
       <c r="AK30" s="21">
         <f t="shared" si="1"/>
@@ -11474,7 +11520,9 @@
       <c r="I31" s="63">
         <v>25.4</v>
       </c>
-      <c r="J31" s="63"/>
+      <c r="J31" s="63">
+        <v>25</v>
+      </c>
       <c r="K31" s="63"/>
       <c r="L31" s="63"/>
       <c r="M31" s="63"/>
@@ -11502,7 +11550,7 @@
       <c r="AI31" s="63"/>
       <c r="AJ31" s="36">
         <f t="shared" si="0"/>
-        <v>25.4</v>
+        <v>25</v>
       </c>
       <c r="AK31" s="21">
         <f t="shared" si="1"/>
@@ -11555,7 +11603,9 @@
       <c r="I32" s="63">
         <v>15.6</v>
       </c>
-      <c r="J32" s="63"/>
+      <c r="J32" s="63">
+        <v>15.6</v>
+      </c>
       <c r="K32" s="63"/>
       <c r="L32" s="63"/>
       <c r="M32" s="63"/>
@@ -11636,7 +11686,9 @@
       <c r="I33" s="63">
         <v>13.8</v>
       </c>
-      <c r="J33" s="63"/>
+      <c r="J33" s="63">
+        <v>14.8</v>
+      </c>
       <c r="K33" s="63"/>
       <c r="L33" s="63"/>
       <c r="M33" s="63"/>
@@ -11664,7 +11716,7 @@
       <c r="AI33" s="63"/>
       <c r="AJ33" s="36">
         <f t="shared" si="0"/>
-        <v>13.8</v>
+        <v>14.8</v>
       </c>
       <c r="AK33" s="21">
         <f t="shared" si="1"/>
@@ -11769,7 +11821,9 @@
       <c r="I35" s="63">
         <v>29.4</v>
       </c>
-      <c r="J35" s="63"/>
+      <c r="J35" s="63">
+        <v>30.6</v>
+      </c>
       <c r="K35" s="63"/>
       <c r="L35" s="63"/>
       <c r="M35" s="63"/>
@@ -11797,7 +11851,7 @@
       <c r="AI35" s="63"/>
       <c r="AJ35" s="36">
         <f t="shared" si="0"/>
-        <v>29.4</v>
+        <v>30.6</v>
       </c>
       <c r="AK35" s="21">
         <f t="shared" si="1"/>
@@ -11971,7 +12025,9 @@
       <c r="I38" s="63">
         <v>31.8</v>
       </c>
-      <c r="J38" s="63"/>
+      <c r="J38" s="63">
+        <v>32.200000000000003</v>
+      </c>
       <c r="K38" s="63"/>
       <c r="L38" s="63"/>
       <c r="M38" s="63"/>
@@ -11999,7 +12055,7 @@
       <c r="AI38" s="63"/>
       <c r="AJ38" s="36">
         <f t="shared" si="0"/>
-        <v>31.8</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="AK38" s="21">
         <f t="shared" si="1"/>
@@ -12053,7 +12109,9 @@
       <c r="I39" s="63">
         <v>32.200000000000003</v>
       </c>
-      <c r="J39" s="63"/>
+      <c r="J39" s="63">
+        <v>32.5</v>
+      </c>
       <c r="K39" s="63"/>
       <c r="L39" s="63"/>
       <c r="M39" s="63"/>
@@ -12081,18 +12139,18 @@
       <c r="AI39" s="63"/>
       <c r="AJ39" s="36">
         <f t="shared" si="0"/>
-        <v>32.200000000000003</v>
+        <v>32.5</v>
       </c>
       <c r="AK39" s="21">
         <f t="shared" si="1"/>
-        <v>32.4</v>
+        <v>32.5</v>
       </c>
       <c r="AL39" s="22">
         <v>36.1</v>
       </c>
       <c r="AM39" s="23">
         <f t="shared" si="2"/>
-        <v>-3.7000000000000028</v>
+        <v>-3.6000000000000014</v>
       </c>
       <c r="AN39" s="23">
         <v>31.513637374860959</v>
@@ -12135,7 +12193,9 @@
       <c r="I40" s="63">
         <v>27.3</v>
       </c>
-      <c r="J40" s="63"/>
+      <c r="J40" s="63">
+        <v>31.2</v>
+      </c>
       <c r="K40" s="63"/>
       <c r="L40" s="63"/>
       <c r="M40" s="63"/>
@@ -12163,7 +12223,7 @@
       <c r="AI40" s="63"/>
       <c r="AJ40" s="36">
         <f t="shared" si="0"/>
-        <v>27.3</v>
+        <v>31.2</v>
       </c>
       <c r="AK40" s="21">
         <f t="shared" si="1"/>
@@ -12217,7 +12277,9 @@
       <c r="I41" s="63">
         <v>30.6</v>
       </c>
-      <c r="J41" s="63"/>
+      <c r="J41" s="63">
+        <v>31.4</v>
+      </c>
       <c r="K41" s="63"/>
       <c r="L41" s="63"/>
       <c r="M41" s="63"/>
@@ -12245,7 +12307,7 @@
       <c r="AI41" s="63"/>
       <c r="AJ41" s="36">
         <f t="shared" si="0"/>
-        <v>30.6</v>
+        <v>31.4</v>
       </c>
       <c r="AK41" s="21">
         <f t="shared" si="1"/>
@@ -12366,7 +12428,9 @@
       <c r="I43" s="63">
         <v>31.8</v>
       </c>
-      <c r="J43" s="63"/>
+      <c r="J43" s="63">
+        <v>32.799999999999997</v>
+      </c>
       <c r="K43" s="63"/>
       <c r="L43" s="63"/>
       <c r="M43" s="63"/>
@@ -12394,18 +12458,18 @@
       <c r="AI43" s="63"/>
       <c r="AJ43" s="36">
         <f t="shared" si="0"/>
-        <v>31.8</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="AK43" s="21">
         <f t="shared" si="1"/>
-        <v>32.200000000000003</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="AL43" s="22">
         <v>35.4</v>
       </c>
       <c r="AM43" s="23">
         <f t="shared" si="2"/>
-        <v>-3.1999999999999957</v>
+        <v>-2.6000000000000014</v>
       </c>
       <c r="AN43" s="23">
         <v>31.022074370307589</v>
@@ -12448,7 +12512,9 @@
       <c r="I44" s="29">
         <v>30.4</v>
       </c>
-      <c r="J44" s="29"/>
+      <c r="J44" s="29">
+        <v>32.200000000000003</v>
+      </c>
       <c r="K44" s="29"/>
       <c r="L44" s="29"/>
       <c r="M44" s="29"/>
@@ -12476,18 +12542,18 @@
       <c r="AI44" s="63"/>
       <c r="AJ44" s="36">
         <f t="shared" si="0"/>
-        <v>30.4</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="AK44" s="21">
         <f t="shared" si="1"/>
-        <v>32</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="AL44" s="22">
         <v>34.4</v>
       </c>
       <c r="AM44" s="23">
         <f t="shared" si="2"/>
-        <v>-2.3999999999999986</v>
+        <v>-2.1999999999999957</v>
       </c>
       <c r="AN44" s="23">
         <v>30.14398006331821</v>
@@ -12530,7 +12596,9 @@
       <c r="I45" s="63">
         <v>29.6</v>
       </c>
-      <c r="J45" s="63"/>
+      <c r="J45" s="63">
+        <v>32.4</v>
+      </c>
       <c r="K45" s="63"/>
       <c r="L45" s="63"/>
       <c r="M45" s="63"/>
@@ -12558,7 +12626,7 @@
       <c r="AI45" s="63"/>
       <c r="AJ45" s="36">
         <f t="shared" si="0"/>
-        <v>29.6</v>
+        <v>32.4</v>
       </c>
       <c r="AK45" s="21">
         <f t="shared" si="1"/>
@@ -12751,7 +12819,9 @@
       <c r="I48" s="63">
         <v>32.5</v>
       </c>
-      <c r="J48" s="63"/>
+      <c r="J48" s="63">
+        <v>31.3</v>
+      </c>
       <c r="K48" s="63"/>
       <c r="L48" s="63"/>
       <c r="M48" s="63"/>
@@ -12779,7 +12849,7 @@
       <c r="AI48" s="63"/>
       <c r="AJ48" s="36">
         <f t="shared" si="0"/>
-        <v>32.5</v>
+        <v>31.3</v>
       </c>
       <c r="AK48" s="21">
         <f t="shared" si="1"/>
@@ -25702,6 +25772,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="N1:N2"/>
     <mergeCell ref="O1:O2"/>
@@ -25711,12 +25787,6 @@
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="L1:L2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:O13 D15:O31 D33:O34 D36:O46">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="equal">

</xml_diff>